<commit_message>
clean up elec/DRC files so that CSV files include HK data
</commit_message>
<xml_diff>
--- a/InputData/elec/DRC/Demand Response Capacity.xlsx
+++ b/InputData/elec/DRC/Demand Response Capacity.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\daiyang.zhang\Desktop\eps-us-3.4.7 HK working\InputData\elec\DRC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mdeng\Desktop\Dropbox_Free_Zone\EPS\Model Repos\China\Subnational\eps-hongkong\InputData\elec\DRC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDE142BA-0100-4B6D-A891-431F5237046D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA525B57-1393-46AF-899C-84B1FF586113}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4515" yWindow="2175" windowWidth="22080" windowHeight="13665" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="Peak Demand Time" sheetId="6" r:id="rId2"/>
     <sheet name="Calculations" sheetId="4" r:id="rId3"/>
     <sheet name="DRC-BDRC" sheetId="5" r:id="rId4"/>
-    <sheet name="DRC-PADRC" sheetId="2" state="hidden" r:id="rId5"/>
+    <sheet name="DRC-PADRC" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,30 +39,8 @@
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="36">
   <si>
     <t>DRC BAU Demand Response Capacity</t>
   </si>
@@ -82,24 +60,9 @@
     <t>periods in response to time-based rates or other financial incentives.</t>
   </si>
   <si>
-    <t>To estimate BAU DR Capacity, we scale Brattle's 2019 estimate of demand response potential by</t>
-  </si>
-  <si>
-    <t>the growth in peak demand (EPS model output).</t>
-  </si>
-  <si>
-    <t>We use a Brattle analysis to estimate the potential in 2030, and scale the potential between 2019 and 2030 linearly.</t>
-  </si>
-  <si>
-    <t>We then scale the potential from 2030 to 2050 by the growth in peak demand (EPS model output).</t>
-  </si>
-  <si>
     <t>Time (Year)</t>
   </si>
   <si>
-    <t>Peak Power Demand after Storage and DR[summer] : MostRecentRun</t>
-  </si>
-  <si>
     <t>Year</t>
   </si>
   <si>
@@ -109,9 +72,6 @@
     <t>Potential Additional DR Capacity (MW)</t>
   </si>
   <si>
-    <t>Peak Demand - EPS Output (CLP)</t>
-  </si>
-  <si>
     <t>https://www.censtatd.gov.hk/en/wbr.html?ecode=B11000022022AN22&amp;scode=90</t>
   </si>
   <si>
@@ -136,29 +96,65 @@
     <t>https://www.censtatd.gov.hk/en/data/stat_report/product/B1100002/att/B11000022021AN21B0100.pdf</t>
   </si>
   <si>
-    <t>Demand Response CLP - Snapshot of CLP in 2022</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://www.clpgroup.com/content/dam/clp-group/channels/media/document/publications/A%20Snapshot%20of%20CLP%20in%202022_Eng.pdf </t>
   </si>
   <si>
     <t>MW reduction</t>
   </si>
   <si>
-    <t>2020 Capacity</t>
-  </si>
-  <si>
-    <t>2050 Projection</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOTE: Although CLP has its own peak demand response capactiy scheme, it has very limited coverage so it is hard to project the demand response forward </t>
+    <t>Peak Hour Electricity Demand by Season[summer] : MostRecentRun</t>
+  </si>
+  <si>
+    <t>Peak Hour Electricity Demand by Season[winter] : MostRecentRun</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/abs/pii/S0142061522007967</t>
+  </si>
+  <si>
+    <t>Wu et al.</t>
+  </si>
+  <si>
+    <t>Maximum demand flexibility from the demand response of a big group of residential homes</t>
+  </si>
+  <si>
+    <t>We assume BAU demand response capacity is zero through 2050.</t>
+  </si>
+  <si>
+    <t>Historical Capacity</t>
+  </si>
+  <si>
+    <t>Future Capacity Projection</t>
+  </si>
+  <si>
+    <t>We use Wu et al.'s assumption that DR can achieve up to a 14.5% in peak demand and linearly scale scale up to this potential in 2030.</t>
+  </si>
+  <si>
+    <t>Although CLP has its own peak demand response capacity scheme, it has very limited coverage so it is hard to project the demand response forward using CLP data.</t>
+  </si>
+  <si>
+    <t>Historical Demand Response - CLP Snapshot in 2022</t>
+  </si>
+  <si>
+    <t>Peak Demand (MW) - EPS Output</t>
+  </si>
+  <si>
+    <t>Future Demand Response</t>
+  </si>
+  <si>
+    <t>% change in summer peak</t>
+  </si>
+  <si>
+    <t>Maximum peak reduction from DR</t>
+  </si>
+  <si>
+    <t>We then hold the potential DR capacity constant from 2031 to 2050.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -189,8 +185,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -209,6 +212,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -219,11 +234,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
@@ -239,10 +255,24 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -312,7 +342,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Peak Demand Time'!$B$4</c:f>
+              <c:f>'Peak Demand Time'!$B$5</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -335,7 +365,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'Peak Demand Time'!$A$5:$A$16</c:f>
+              <c:f>'Peak Demand Time'!$A$6:$A$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
@@ -380,7 +410,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Peak Demand Time'!$B$5:$B$16</c:f>
+              <c:f>'Peak Demand Time'!$B$6:$B$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
@@ -1156,13 +1186,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>819150</xdr:colOff>
-      <xdr:row>2</xdr:row>
+      <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>812800</xdr:colOff>
-      <xdr:row>21</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>165100</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1478,313 +1508,344 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B27"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B30"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="28.453125" customWidth="1"/>
+    <col min="2" max="2" width="28.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B6" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B8" s="6" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B5" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B10" s="13">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B12" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B8" s="6" t="s">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="1"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="12"/>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="12" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" s="1"/>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B26" s="1"/>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B27" s="3"/>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="14">
+        <v>0.14499999999999999</v>
+      </c>
+      <c r="B24" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B29" s="1"/>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B30" s="3"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B12" r:id="rId1" xr:uid="{08A4D078-1C2D-454E-852F-D6FD41D542C0}"/>
+    <hyperlink ref="B6" r:id="rId2" xr:uid="{C3B2D2A1-804A-474E-8F67-34ABE7C47B78}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61617D0E-654C-384D-A408-E7E11AE547D1}">
-  <dimension ref="A1:D24"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="9"/>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="9"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
+        <v>11</v>
+      </c>
       <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
       <c r="D3" s="9"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>18</v>
-      </c>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="9">
-        <v>2011</v>
-      </c>
-      <c r="B5" s="9">
-        <v>10296</v>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>12</v>
       </c>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="9">
-        <v>2012</v>
+        <v>2011</v>
       </c>
       <c r="B6" s="9">
-        <v>9925</v>
+        <v>10296</v>
       </c>
       <c r="C6" s="9"/>
       <c r="D6" s="9"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="9">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="B7" s="9">
-        <v>10068</v>
+        <v>9925</v>
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="B8" s="9">
-        <v>9962</v>
+        <v>10068</v>
       </c>
       <c r="C8" s="9"/>
       <c r="D8" s="9"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="9">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="B9" s="9">
-        <v>10009</v>
+        <v>9962</v>
       </c>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
-        <v>2016</v>
+        <v>2015</v>
       </c>
       <c r="B10" s="9">
-        <v>9937</v>
+        <v>10009</v>
       </c>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="9">
-        <v>2017</v>
+        <v>2016</v>
       </c>
       <c r="B11" s="9">
-        <v>10696</v>
+        <v>9937</v>
       </c>
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="9">
-        <v>2018</v>
+        <v>2017</v>
       </c>
       <c r="B12" s="9">
-        <v>9692</v>
+        <v>10696</v>
       </c>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="9">
-        <v>2019</v>
+        <v>2018</v>
       </c>
       <c r="B13" s="9">
-        <v>9601</v>
+        <v>9692</v>
       </c>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="9">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="B14" s="9">
-        <v>9670</v>
+        <v>9601</v>
       </c>
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="9">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="B15" s="9">
-        <v>9942</v>
+        <v>9670</v>
       </c>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="9">
-        <v>2022</v>
-      </c>
-      <c r="B16">
-        <v>10104</v>
+        <v>2021</v>
+      </c>
+      <c r="B16" s="9">
+        <v>9942</v>
       </c>
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" s="9"/>
-      <c r="B17" s="9"/>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="9">
+        <v>2022</v>
+      </c>
+      <c r="B17">
+        <v>10104</v>
+      </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="9">
-        <f>AVERAGE(B5:B16)</f>
-        <v>9991.8333333333339</v>
-      </c>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="9"/>
+      <c r="B18" s="9"/>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" s="9"/>
-      <c r="B19" s="9"/>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B19" s="9">
+        <f>AVERAGE(B6:B17)</f>
+        <v>9991.8333333333339</v>
+      </c>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="9"/>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="9"/>
       <c r="B21" s="9"/>
       <c r="C21" s="9"/>
       <c r="D21" s="9"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="9"/>
       <c r="B22" s="9"/>
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A23" s="9" t="s">
-        <v>20</v>
-      </c>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="9"/>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B24" s="9"/>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1794,264 +1855,709 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AH9"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetPr>
+    <pageSetUpPr autoPageBreaks="0"/>
+  </sheetPr>
+  <dimension ref="A1:AH20"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="1" max="1" width="44.85546875" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:34" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="8"/>
+    </row>
+    <row r="2" spans="1:34" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3">
+        <v>2021</v>
+      </c>
+      <c r="C3">
+        <v>2022</v>
+      </c>
+      <c r="D3">
+        <v>2023</v>
+      </c>
+      <c r="E3">
+        <v>2024</v>
+      </c>
+      <c r="F3">
+        <v>2025</v>
+      </c>
+      <c r="G3">
+        <v>2026</v>
+      </c>
+      <c r="H3">
+        <v>2027</v>
+      </c>
+      <c r="I3">
+        <v>2028</v>
+      </c>
+      <c r="J3">
+        <v>2029</v>
+      </c>
+      <c r="K3">
+        <v>2030</v>
+      </c>
+      <c r="L3">
+        <v>2031</v>
+      </c>
+      <c r="M3">
+        <v>2032</v>
+      </c>
+      <c r="N3">
+        <v>2033</v>
+      </c>
+      <c r="O3">
+        <v>2034</v>
+      </c>
+      <c r="P3">
+        <v>2035</v>
+      </c>
+      <c r="Q3">
+        <v>2036</v>
+      </c>
+      <c r="R3">
+        <v>2037</v>
+      </c>
+      <c r="S3">
+        <v>2038</v>
+      </c>
+      <c r="T3">
+        <v>2039</v>
+      </c>
+      <c r="U3">
+        <v>2040</v>
+      </c>
+      <c r="V3">
+        <v>2041</v>
+      </c>
+      <c r="W3">
+        <v>2042</v>
+      </c>
+      <c r="X3">
+        <v>2043</v>
+      </c>
+      <c r="Y3">
+        <v>2044</v>
+      </c>
+      <c r="Z3">
+        <v>2045</v>
+      </c>
+      <c r="AA3">
+        <v>2046</v>
+      </c>
+      <c r="AB3">
+        <v>2047</v>
+      </c>
+      <c r="AC3">
+        <v>2048</v>
+      </c>
+      <c r="AD3">
+        <v>2049</v>
+      </c>
+      <c r="AE3">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="4" spans="1:34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4">
+        <v>10185.9</v>
+      </c>
+      <c r="C4">
+        <v>10567.3</v>
+      </c>
+      <c r="D4">
+        <v>10624.7</v>
+      </c>
+      <c r="E4">
+        <v>10778.6</v>
+      </c>
+      <c r="F4">
+        <v>10972.3</v>
+      </c>
+      <c r="G4">
+        <v>11066.3</v>
+      </c>
+      <c r="H4">
+        <v>11122.6</v>
+      </c>
+      <c r="I4">
+        <v>11182.8</v>
+      </c>
+      <c r="J4">
+        <v>11258.7</v>
+      </c>
+      <c r="K4">
+        <v>11309.6</v>
+      </c>
+      <c r="L4">
+        <v>11370.6</v>
+      </c>
+      <c r="M4">
+        <v>11409</v>
+      </c>
+      <c r="N4">
+        <v>11381.4</v>
+      </c>
+      <c r="O4">
+        <v>11334.7</v>
+      </c>
+      <c r="P4">
+        <v>11294.8</v>
+      </c>
+      <c r="Q4">
+        <v>10299</v>
+      </c>
+      <c r="R4">
+        <v>17292.7</v>
+      </c>
+      <c r="S4">
+        <v>12631.9</v>
+      </c>
+      <c r="T4">
+        <v>11373.7</v>
+      </c>
+      <c r="U4">
+        <v>7995.37</v>
+      </c>
+      <c r="V4">
+        <v>14627.4</v>
+      </c>
+      <c r="W4">
+        <v>12294.1</v>
+      </c>
+      <c r="X4">
+        <v>10572.5</v>
+      </c>
+      <c r="Y4">
+        <v>20810.400000000001</v>
+      </c>
+      <c r="Z4">
+        <v>13595.5</v>
+      </c>
+      <c r="AA4">
+        <v>11349.6</v>
+      </c>
+      <c r="AB4">
+        <v>23934.6</v>
+      </c>
+      <c r="AC4">
+        <v>13708.6</v>
+      </c>
+      <c r="AD4">
+        <v>10064.299999999999</v>
+      </c>
+      <c r="AE4">
+        <v>21318.6</v>
+      </c>
+      <c r="AH4" s="7"/>
+    </row>
+    <row r="5" spans="1:34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5">
+        <v>4260.49</v>
+      </c>
+      <c r="C5">
+        <v>4918.7299999999996</v>
+      </c>
+      <c r="D5">
+        <v>5012.6899999999996</v>
+      </c>
+      <c r="E5">
+        <v>5143.4399999999996</v>
+      </c>
+      <c r="F5">
+        <v>5301.45</v>
+      </c>
+      <c r="G5">
+        <v>5408.32</v>
+      </c>
+      <c r="H5">
+        <v>5501.93</v>
+      </c>
+      <c r="I5">
+        <v>5580.31</v>
+      </c>
+      <c r="J5">
+        <v>5667.82</v>
+      </c>
+      <c r="K5">
+        <v>5748.58</v>
+      </c>
+      <c r="L5">
+        <v>5822.41</v>
+      </c>
+      <c r="M5">
+        <v>5881.54</v>
+      </c>
+      <c r="N5">
+        <v>5903.72</v>
+      </c>
+      <c r="O5">
+        <v>5900.18</v>
+      </c>
+      <c r="P5">
+        <v>5937.77</v>
+      </c>
+      <c r="Q5">
+        <v>5503.24</v>
+      </c>
+      <c r="R5">
+        <v>9567.31</v>
+      </c>
+      <c r="S5">
+        <v>6890.15</v>
+      </c>
+      <c r="T5">
+        <v>6147.6</v>
+      </c>
+      <c r="U5">
+        <v>4205.6499999999996</v>
+      </c>
+      <c r="V5">
+        <v>8179.5</v>
+      </c>
+      <c r="W5">
+        <v>6822.99</v>
+      </c>
+      <c r="X5">
+        <v>5818.31</v>
+      </c>
+      <c r="Y5">
+        <v>12434.1</v>
+      </c>
+      <c r="Z5">
+        <v>7474.48</v>
+      </c>
+      <c r="AA5">
+        <v>5969.17</v>
+      </c>
+      <c r="AB5">
+        <v>14885.3</v>
+      </c>
+      <c r="AC5">
+        <v>7079.23</v>
+      </c>
+      <c r="AD5">
+        <v>5260.41</v>
+      </c>
+      <c r="AE5">
+        <v>12946.9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:34" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="1:34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="16">
+        <f>(C4-B4)/B4</f>
+        <v>3.7443917572330343E-2</v>
+      </c>
+      <c r="D7" s="16">
+        <f t="shared" ref="D7:AE7" si="0">(D4-C4)/C4</f>
+        <v>5.4318510877898289E-3</v>
+      </c>
+      <c r="E7" s="16">
+        <f t="shared" si="0"/>
+        <v>1.4485114873831697E-2</v>
+      </c>
+      <c r="F7" s="16">
+        <f t="shared" si="0"/>
+        <v>1.7970793980665291E-2</v>
+      </c>
+      <c r="G7" s="16">
+        <f t="shared" si="0"/>
+        <v>8.5670278792960453E-3</v>
+      </c>
+      <c r="H7" s="16">
+        <f t="shared" si="0"/>
+        <v>5.0875179599325065E-3</v>
+      </c>
+      <c r="I7" s="16">
+        <f t="shared" si="0"/>
+        <v>5.4124035747036576E-3</v>
+      </c>
+      <c r="J7" s="16">
+        <f t="shared" si="0"/>
+        <v>6.7872089279966972E-3</v>
+      </c>
+      <c r="K7" s="16">
+        <f t="shared" si="0"/>
+        <v>4.5209482444686895E-3</v>
+      </c>
+      <c r="L7" s="16">
+        <f t="shared" si="0"/>
+        <v>5.3936478743722149E-3</v>
+      </c>
+      <c r="M7" s="16">
+        <f t="shared" si="0"/>
+        <v>3.3771304944329793E-3</v>
+      </c>
+      <c r="N7" s="16">
+        <f t="shared" si="0"/>
+        <v>-2.4191427820142311E-3</v>
+      </c>
+      <c r="O7" s="16">
+        <f t="shared" si="0"/>
+        <v>-4.1031858998013346E-3</v>
+      </c>
+      <c r="P7" s="16">
+        <f t="shared" si="0"/>
+        <v>-3.5201637449602946E-3</v>
+      </c>
+      <c r="Q7" s="16">
+        <f t="shared" si="0"/>
+        <v>-8.8164465063569022E-2</v>
+      </c>
+      <c r="R7" s="16">
+        <f t="shared" si="0"/>
+        <v>0.67906592873094485</v>
+      </c>
+      <c r="S7" s="16">
+        <f t="shared" si="0"/>
+        <v>-0.26952413446136236</v>
+      </c>
+      <c r="T7" s="16">
+        <f t="shared" si="0"/>
+        <v>-9.9604968373720418E-2</v>
+      </c>
+      <c r="U7" s="16">
+        <f t="shared" si="0"/>
+        <v>-0.29702999024064292</v>
+      </c>
+      <c r="V7" s="16">
+        <f t="shared" si="0"/>
+        <v>0.82948381375721192</v>
+      </c>
+      <c r="W7" s="16">
+        <f t="shared" si="0"/>
+        <v>-0.15951570340593677</v>
+      </c>
+      <c r="X7" s="16">
+        <f t="shared" si="0"/>
+        <v>-0.14003465076744132</v>
+      </c>
+      <c r="Y7" s="16">
+        <f t="shared" si="0"/>
+        <v>0.96835185623078757</v>
+      </c>
+      <c r="Z7" s="16">
+        <f t="shared" si="0"/>
+        <v>-0.34669684388574951</v>
+      </c>
+      <c r="AA7" s="16">
+        <f t="shared" si="0"/>
+        <v>-0.16519436578279575</v>
+      </c>
+      <c r="AB7" s="16">
+        <f t="shared" si="0"/>
+        <v>1.1088496510890249</v>
+      </c>
+      <c r="AC7" s="16">
+        <f t="shared" si="0"/>
+        <v>-0.42724758299700011</v>
+      </c>
+      <c r="AD7" s="16">
+        <f t="shared" si="0"/>
+        <v>-0.26584042134134783</v>
+      </c>
+      <c r="AE7" s="16">
+        <f t="shared" si="0"/>
+        <v>1.118239718609342</v>
+      </c>
+    </row>
+    <row r="9" spans="1:34" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="8"/>
+    </row>
+    <row r="10" spans="1:34" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C2">
+    </row>
+    <row r="11" spans="1:34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E11" s="2"/>
+    </row>
+    <row r="13" spans="1:34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C13" s="10">
+        <v>2019</v>
+      </c>
+      <c r="D13" s="10">
         <v>2020</v>
       </c>
-      <c r="D2">
+      <c r="E13" s="10">
         <v>2021</v>
       </c>
-      <c r="E2">
+      <c r="F13" s="10">
         <v>2022</v>
       </c>
-      <c r="F2">
+    </row>
+    <row r="14" spans="1:34" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14">
+        <v>118</v>
+      </c>
+      <c r="D14">
+        <v>104</v>
+      </c>
+      <c r="E14">
+        <v>70</v>
+      </c>
+      <c r="F14">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="16" spans="1:34" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="8"/>
+    </row>
+    <row r="18" spans="1:31" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B18">
+        <v>2021</v>
+      </c>
+      <c r="C18">
+        <v>2022</v>
+      </c>
+      <c r="D18">
         <v>2023</v>
       </c>
-      <c r="G2">
+      <c r="E18">
         <v>2024</v>
       </c>
-      <c r="H2">
+      <c r="F18">
         <v>2025</v>
       </c>
-      <c r="I2">
+      <c r="G18">
         <v>2026</v>
       </c>
-      <c r="J2">
+      <c r="H18">
         <v>2027</v>
       </c>
-      <c r="K2">
+      <c r="I18">
         <v>2028</v>
       </c>
-      <c r="L2">
+      <c r="J18">
         <v>2029</v>
       </c>
-      <c r="M2">
+      <c r="K18">
         <v>2030</v>
       </c>
-      <c r="N2">
+      <c r="L18">
         <v>2031</v>
       </c>
-      <c r="O2">
+      <c r="M18">
         <v>2032</v>
       </c>
-      <c r="P2">
+      <c r="N18">
         <v>2033</v>
       </c>
-      <c r="Q2">
+      <c r="O18">
         <v>2034</v>
       </c>
-      <c r="R2">
+      <c r="P18">
         <v>2035</v>
       </c>
-      <c r="S2">
+      <c r="Q18">
         <v>2036</v>
       </c>
-      <c r="T2">
+      <c r="R18">
         <v>2037</v>
       </c>
-      <c r="U2">
+      <c r="S18">
         <v>2038</v>
       </c>
-      <c r="V2">
+      <c r="T18">
         <v>2039</v>
       </c>
-      <c r="W2">
+      <c r="U18">
         <v>2040</v>
       </c>
-      <c r="X2">
+      <c r="V18">
         <v>2041</v>
       </c>
-      <c r="Y2">
+      <c r="W18">
         <v>2042</v>
       </c>
-      <c r="Z2">
+      <c r="X18">
         <v>2043</v>
       </c>
-      <c r="AA2">
+      <c r="Y18">
         <v>2044</v>
       </c>
-      <c r="AB2">
+      <c r="Z18">
         <v>2045</v>
       </c>
-      <c r="AC2">
+      <c r="AA18">
         <v>2046</v>
       </c>
-      <c r="AD2">
+      <c r="AB18">
         <v>2047</v>
       </c>
-      <c r="AE2">
+      <c r="AC18">
         <v>2048</v>
       </c>
-      <c r="AF2">
+      <c r="AD18">
         <v>2049</v>
       </c>
-      <c r="AG2">
+      <c r="AE18">
         <v>2050</v>
       </c>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3">
-        <v>9670</v>
-      </c>
-      <c r="D3">
-        <v>9942</v>
-      </c>
-      <c r="E3">
-        <v>10104</v>
-      </c>
-      <c r="F3" cm="1">
-        <f t="array" ref="F3:AG3">TREND(C3:E3,C2:E2,F2:AG2)</f>
-        <v>10339.333333333314</v>
-      </c>
-      <c r="G3">
-        <v>10556.333333333314</v>
-      </c>
-      <c r="H3">
-        <v>10773.333333333314</v>
-      </c>
-      <c r="I3">
-        <v>10990.333333333314</v>
-      </c>
-      <c r="J3">
-        <v>11207.333333333314</v>
-      </c>
-      <c r="K3">
-        <v>11424.333333333314</v>
-      </c>
-      <c r="L3">
-        <v>11641.333333333314</v>
-      </c>
-      <c r="M3">
-        <v>11858.333333333314</v>
-      </c>
-      <c r="N3">
-        <v>12075.333333333314</v>
-      </c>
-      <c r="O3">
-        <v>12292.333333333314</v>
-      </c>
-      <c r="P3">
-        <v>12509.333333333314</v>
-      </c>
-      <c r="Q3">
-        <v>12726.333333333314</v>
-      </c>
-      <c r="R3">
-        <v>12943.333333333314</v>
-      </c>
-      <c r="S3">
-        <v>13160.333333333314</v>
-      </c>
-      <c r="T3">
-        <v>13377.333333333314</v>
-      </c>
-      <c r="U3">
-        <v>13594.333333333314</v>
-      </c>
-      <c r="V3">
-        <v>13811.333333333314</v>
-      </c>
-      <c r="W3">
-        <v>14028.333333333314</v>
-      </c>
-      <c r="X3">
-        <v>14245.333333333314</v>
-      </c>
-      <c r="Y3">
-        <v>14462.333333333314</v>
-      </c>
-      <c r="Z3">
-        <v>14679.333333333314</v>
-      </c>
-      <c r="AA3">
-        <v>14896.333333333314</v>
-      </c>
-      <c r="AB3">
-        <v>15113.333333333314</v>
-      </c>
-      <c r="AC3">
-        <v>15330.333333333314</v>
-      </c>
-      <c r="AD3">
-        <v>15547.333333333314</v>
-      </c>
-      <c r="AE3">
-        <v>15764.333333333314</v>
-      </c>
-      <c r="AF3">
-        <v>15981.333333333314</v>
-      </c>
-      <c r="AG3">
-        <v>16198.333333333314</v>
-      </c>
-      <c r="AH3" s="7"/>
-    </row>
-    <row r="6" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="C8" s="10">
-        <v>2019</v>
-      </c>
-      <c r="D8" s="10">
-        <v>2020</v>
-      </c>
-      <c r="E8" s="10">
-        <v>2021</v>
-      </c>
-      <c r="F8" s="10">
-        <v>2022</v>
-      </c>
-    </row>
-    <row r="9" spans="1:34" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9">
-        <v>118</v>
-      </c>
-      <c r="D9">
-        <v>104</v>
-      </c>
-      <c r="E9">
+    <row r="19" spans="1:31" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="15">
+        <f>E14</f>
         <v>70</v>
       </c>
-      <c r="F9">
+      <c r="C19" s="15">
+        <f>F14</f>
         <v>130</v>
       </c>
-    </row>
+      <c r="D19" s="4">
+        <f>($K$19-$C$19)/COUNT($D$18:$K$18)+C19</f>
+        <v>318.73649999999998</v>
+      </c>
+      <c r="E19" s="4">
+        <f t="shared" ref="E19:J19" si="1">($K$19-$C$19)/COUNT($D$18:$K$18)+D19</f>
+        <v>507.47299999999996</v>
+      </c>
+      <c r="F19" s="4">
+        <f t="shared" si="1"/>
+        <v>696.20949999999993</v>
+      </c>
+      <c r="G19" s="4">
+        <f t="shared" si="1"/>
+        <v>884.94599999999991</v>
+      </c>
+      <c r="H19" s="4">
+        <f t="shared" si="1"/>
+        <v>1073.6824999999999</v>
+      </c>
+      <c r="I19" s="4">
+        <f t="shared" si="1"/>
+        <v>1262.4189999999999</v>
+      </c>
+      <c r="J19" s="4">
+        <f t="shared" si="1"/>
+        <v>1451.1554999999998</v>
+      </c>
+      <c r="K19" s="17">
+        <f>About!$A$24*K4</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="L19" s="18">
+        <f>K19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="M19" s="18">
+        <f t="shared" ref="M19:AE19" si="2">L19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="N19" s="18">
+        <f t="shared" si="2"/>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="O19" s="18">
+        <f t="shared" si="2"/>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="P19" s="18">
+        <f t="shared" si="2"/>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="Q19" s="18">
+        <f t="shared" si="2"/>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="R19" s="18">
+        <f t="shared" si="2"/>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="S19" s="18">
+        <f t="shared" si="2"/>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="T19" s="18">
+        <f t="shared" si="2"/>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="U19" s="18">
+        <f t="shared" si="2"/>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="V19" s="18">
+        <f t="shared" si="2"/>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="W19" s="18">
+        <f t="shared" si="2"/>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="X19" s="18">
+        <f t="shared" si="2"/>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="Y19" s="18">
+        <f t="shared" si="2"/>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="Z19" s="18">
+        <f t="shared" si="2"/>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="AA19" s="18">
+        <f t="shared" si="2"/>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="AB19" s="18">
+        <f t="shared" si="2"/>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="AC19" s="18">
+        <f t="shared" si="2"/>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="AD19" s="18">
+        <f t="shared" si="2"/>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="AE19" s="18">
+        <f t="shared" si="2"/>
+        <v>1639.8920000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:31" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C1" r:id="rId1" xr:uid="{B8B6E743-3535-B242-AD51-586DF3E76FC3}"/>
-    <hyperlink ref="E6" r:id="rId2" xr:uid="{E4B16B2A-F24C-074A-A8EC-4FFFA6E30104}"/>
+    <hyperlink ref="A11" r:id="rId1" xr:uid="{E4B16B2A-F24C-074A-A8EC-4FFFA6E30104}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -2060,113 +2566,110 @@
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AE2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.36328125" customWidth="1"/>
+    <col min="1" max="1" width="19.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B1">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C1">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="D1">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="E1">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F1">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="G1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="H1">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="I1">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="J1">
-        <v>2028</v>
+        <v>2029</v>
       </c>
       <c r="K1">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="L1">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="M1">
-        <v>2031</v>
+        <v>2032</v>
       </c>
       <c r="N1">
-        <v>2032</v>
+        <v>2033</v>
       </c>
       <c r="O1">
-        <v>2033</v>
+        <v>2034</v>
       </c>
       <c r="P1">
-        <v>2034</v>
+        <v>2035</v>
       </c>
       <c r="Q1">
-        <v>2035</v>
+        <v>2036</v>
       </c>
       <c r="R1">
-        <v>2036</v>
+        <v>2037</v>
       </c>
       <c r="S1">
-        <v>2037</v>
+        <v>2038</v>
       </c>
       <c r="T1">
-        <v>2038</v>
+        <v>2039</v>
       </c>
       <c r="U1">
-        <v>2039</v>
+        <v>2040</v>
       </c>
       <c r="V1">
-        <v>2040</v>
+        <v>2041</v>
       </c>
       <c r="W1">
-        <v>2041</v>
+        <v>2042</v>
       </c>
       <c r="X1">
-        <v>2042</v>
+        <v>2043</v>
       </c>
       <c r="Y1">
-        <v>2043</v>
+        <v>2044</v>
       </c>
       <c r="Z1">
-        <v>2044</v>
+        <v>2045</v>
       </c>
       <c r="AA1">
-        <v>2045</v>
+        <v>2046</v>
       </c>
       <c r="AB1">
-        <v>2046</v>
+        <v>2047</v>
       </c>
       <c r="AC1">
-        <v>2047</v>
+        <v>2048</v>
       </c>
       <c r="AD1">
-        <v>2048</v>
+        <v>2049</v>
       </c>
       <c r="AE1">
-        <v>2049</v>
-      </c>
-      <c r="AF1">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B2" s="9">
         <v>0</v>
@@ -2256,9 +2759,6 @@
         <v>0</v>
       </c>
       <c r="AE2" s="9">
-        <v>0</v>
-      </c>
-      <c r="AF2" s="9">
         <v>0</v>
       </c>
     </row>
@@ -2272,251 +2772,230 @@
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AH2"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AE2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B1">
-        <v>2018</v>
+        <v>2021</v>
       </c>
       <c r="C1">
-        <v>2019</v>
+        <v>2022</v>
       </c>
       <c r="D1">
-        <v>2020</v>
+        <v>2023</v>
       </c>
       <c r="E1">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="F1">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="G1">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="H1">
-        <v>2024</v>
+        <v>2027</v>
       </c>
       <c r="I1">
-        <v>2025</v>
+        <v>2028</v>
       </c>
       <c r="J1">
-        <v>2026</v>
+        <v>2029</v>
       </c>
       <c r="K1">
-        <v>2027</v>
+        <v>2030</v>
       </c>
       <c r="L1">
-        <v>2028</v>
+        <v>2031</v>
       </c>
       <c r="M1">
-        <v>2029</v>
+        <v>2032</v>
       </c>
       <c r="N1">
-        <v>2030</v>
+        <v>2033</v>
       </c>
       <c r="O1">
-        <v>2031</v>
+        <v>2034</v>
       </c>
       <c r="P1">
-        <v>2032</v>
+        <v>2035</v>
       </c>
       <c r="Q1">
-        <v>2033</v>
+        <v>2036</v>
       </c>
       <c r="R1">
-        <v>2034</v>
+        <v>2037</v>
       </c>
       <c r="S1">
-        <v>2035</v>
+        <v>2038</v>
       </c>
       <c r="T1">
-        <v>2036</v>
+        <v>2039</v>
       </c>
       <c r="U1">
-        <v>2037</v>
+        <v>2040</v>
       </c>
       <c r="V1">
-        <v>2038</v>
+        <v>2041</v>
       </c>
       <c r="W1">
-        <v>2039</v>
+        <v>2042</v>
       </c>
       <c r="X1">
-        <v>2040</v>
+        <v>2043</v>
       </c>
       <c r="Y1">
-        <v>2041</v>
+        <v>2044</v>
       </c>
       <c r="Z1">
-        <v>2042</v>
+        <v>2045</v>
       </c>
       <c r="AA1">
-        <v>2043</v>
+        <v>2046</v>
       </c>
       <c r="AB1">
-        <v>2044</v>
+        <v>2047</v>
       </c>
       <c r="AC1">
-        <v>2045</v>
+        <v>2048</v>
       </c>
       <c r="AD1">
-        <v>2046</v>
+        <v>2049</v>
       </c>
       <c r="AE1">
-        <v>2047</v>
-      </c>
-      <c r="AF1">
-        <v>2048</v>
-      </c>
-      <c r="AG1">
-        <v>2049</v>
-      </c>
-      <c r="AH1">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:34" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="4" t="e">
-        <f>C2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="C2" s="4" t="e">
-        <f>Calculations!#REF!-'DRC-BDRC'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!D1)-'DRC-BDRC'!B2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!E1)-'DRC-BDRC'!C2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!F1)-'DRC-BDRC'!D2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!G1)-'DRC-BDRC'!E2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!H1)-'DRC-BDRC'!F2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="I2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!I1)-'DRC-BDRC'!G2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="J2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!J1)-'DRC-BDRC'!H2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!K1)-'DRC-BDRC'!I2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!L1)-'DRC-BDRC'!J2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="M2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!M1)-'DRC-BDRC'!K2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="N2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!N1)-'DRC-BDRC'!L2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="O2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!O1)-'DRC-BDRC'!M2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="P2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!P1)-'DRC-BDRC'!N2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Q2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!Q1)-'DRC-BDRC'!O2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="R2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!R1)-'DRC-BDRC'!P2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="S2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!S1)-'DRC-BDRC'!Q2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="T2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!T1)-'DRC-BDRC'!R2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="U2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!U1)-'DRC-BDRC'!S2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="V2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!V1)-'DRC-BDRC'!T2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="W2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!W1)-'DRC-BDRC'!U2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="X2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!X1)-'DRC-BDRC'!V2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Y2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!Y1)-'DRC-BDRC'!W2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="Z2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!Z1)-'DRC-BDRC'!X2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="AA2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!AA1)-'DRC-BDRC'!Y2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="AB2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!AB1)-'DRC-BDRC'!Z2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="AC2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!AC1)-'DRC-BDRC'!AA2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="AD2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!AD1)-'DRC-BDRC'!AB2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="AE2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!AE1)-'DRC-BDRC'!AC2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="AF2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!AF1)-'DRC-BDRC'!AD2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="AG2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!AG1)-'DRC-BDRC'!AE2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="AH2" s="4" t="e">
-        <f>TREND(Calculations!#REF!,Calculations!#REF!,'DRC-PADRC'!AH1)-'DRC-BDRC'!AF2</f>
-        <v>#REF!</v>
+        <v>9</v>
+      </c>
+      <c r="B2" s="19">
+        <f>Calculations!B19</f>
+        <v>70</v>
+      </c>
+      <c r="C2" s="19">
+        <f>Calculations!C19</f>
+        <v>130</v>
+      </c>
+      <c r="D2" s="19">
+        <f>Calculations!D19</f>
+        <v>318.73649999999998</v>
+      </c>
+      <c r="E2" s="19">
+        <f>Calculations!E19</f>
+        <v>507.47299999999996</v>
+      </c>
+      <c r="F2" s="19">
+        <f>Calculations!F19</f>
+        <v>696.20949999999993</v>
+      </c>
+      <c r="G2" s="19">
+        <f>Calculations!G19</f>
+        <v>884.94599999999991</v>
+      </c>
+      <c r="H2" s="19">
+        <f>Calculations!H19</f>
+        <v>1073.6824999999999</v>
+      </c>
+      <c r="I2" s="19">
+        <f>Calculations!I19</f>
+        <v>1262.4189999999999</v>
+      </c>
+      <c r="J2" s="19">
+        <f>Calculations!J19</f>
+        <v>1451.1554999999998</v>
+      </c>
+      <c r="K2" s="19">
+        <f>Calculations!K19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="L2" s="19">
+        <f>Calculations!L19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="M2" s="19">
+        <f>Calculations!M19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="N2" s="19">
+        <f>Calculations!N19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="O2" s="19">
+        <f>Calculations!O19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="P2" s="19">
+        <f>Calculations!P19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="Q2" s="19">
+        <f>Calculations!Q19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="R2" s="19">
+        <f>Calculations!R19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="S2" s="19">
+        <f>Calculations!S19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="T2" s="19">
+        <f>Calculations!T19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="U2" s="19">
+        <f>Calculations!U19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="V2" s="19">
+        <f>Calculations!V19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="W2" s="19">
+        <f>Calculations!W19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="X2" s="19">
+        <f>Calculations!X19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="Y2" s="19">
+        <f>Calculations!Y19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="Z2" s="19">
+        <f>Calculations!Z19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="AA2" s="19">
+        <f>Calculations!AA19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="AB2" s="19">
+        <f>Calculations!AB19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="AC2" s="19">
+        <f>Calculations!AC19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="AD2" s="19">
+        <f>Calculations!AD19</f>
+        <v>1639.8920000000001</v>
+      </c>
+      <c r="AE2" s="19">
+        <f>Calculations!AE19</f>
+        <v>1639.8920000000001</v>
       </c>
     </row>
   </sheetData>
@@ -2525,15 +3004,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D257B2780BAD0A45A02FA065B9C6CC6A" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="54b727ac31dab95898e9cf92f0402afe">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cb176f07-3112-4ee9-93fd-ae2cb5f3e433" xmlns:ns3="6b15a3a4-8173-42d6-9deb-398ec38eca4b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="42611c3eb46fef4c2b2610d1e51cc1b0" ns2:_="" ns3:_="">
     <xsd:import namespace="cb176f07-3112-4ee9-93fd-ae2cb5f3e433"/>
@@ -2782,15 +3252,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C9688730-E746-4F6D-A8FC-7D3E96F062FE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FA69326-0AE3-4ED9-B194-0C025F2DBE0A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2807,4 +3278,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C9688730-E746-4F6D-A8FC-7D3E96F062FE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>